<commit_message>
chore(weekly-sync): auto-pull through 2026-06-02
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week22.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week22.xlsx
@@ -482,10 +482,10 @@
         <v>13820</v>
       </c>
       <c r="G2" t="n">
-        <v>9785.58</v>
+        <v>13047.44</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -566,10 +566,10 @@
         <v>11806</v>
       </c>
       <c r="G5" t="n">
-        <v>2540.68</v>
+        <v>3909.32</v>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -594,10 +594,10 @@
         <v>16289</v>
       </c>
       <c r="G6" t="n">
-        <v>6775.4</v>
+        <v>8130.48</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -675,7 +675,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -703,7 +703,7 @@
         <v>16</v>
       </c>
       <c r="F10" t="n">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="G10" t="n">
         <v>7964.4</v>
@@ -787,7 +787,7 @@
         <v>54</v>
       </c>
       <c r="F13" t="n">
-        <v>14929</v>
+        <v>14927</v>
       </c>
       <c r="G13" t="n">
         <v>8471.200000000001</v>
@@ -815,7 +815,7 @@
         <v>31</v>
       </c>
       <c r="F14" t="n">
-        <v>7748</v>
+        <v>7747</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -874,10 +874,10 @@
         <v>4714</v>
       </c>
       <c r="G16" t="n">
-        <v>23133.05</v>
+        <v>30759.32</v>
       </c>
       <c r="H16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -1011,7 +1011,7 @@
         <v>269</v>
       </c>
       <c r="F21" t="n">
-        <v>46443</v>
+        <v>46442</v>
       </c>
       <c r="G21" t="n">
         <v>6310.17</v>
@@ -1434,10 +1434,10 @@
         <v>17690</v>
       </c>
       <c r="G36" t="n">
-        <v>13835.49</v>
+        <v>18325.33</v>
       </c>
       <c r="H36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -1627,7 +1627,7 @@
         <v>100</v>
       </c>
       <c r="F43" t="n">
-        <v>22699</v>
+        <v>22698</v>
       </c>
       <c r="G43" t="n">
         <v>6438.98</v>
@@ -1795,7 +1795,7 @@
         <v>101</v>
       </c>
       <c r="F49" t="n">
-        <v>27545</v>
+        <v>27543</v>
       </c>
       <c r="G49" t="n">
         <v>1647.46</v>
@@ -2019,7 +2019,7 @@
         <v>282</v>
       </c>
       <c r="F57" t="n">
-        <v>84307</v>
+        <v>84306</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -2187,13 +2187,13 @@
         <v>900</v>
       </c>
       <c r="F63" t="n">
-        <v>111315</v>
+        <v>111313</v>
       </c>
       <c r="G63" t="n">
-        <v>66256.76000000001</v>
+        <v>74390.66</v>
       </c>
       <c r="H63" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="64">
@@ -2277,7 +2277,7 @@
         <v>49633.91</v>
       </c>
       <c r="H66" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67">
@@ -2495,7 +2495,7 @@
         <v>254</v>
       </c>
       <c r="F74" t="n">
-        <v>40686</v>
+        <v>40685</v>
       </c>
       <c r="G74" t="n">
         <v>17069.52</v>
@@ -2803,7 +2803,7 @@
         <v>373</v>
       </c>
       <c r="F85" t="n">
-        <v>51448</v>
+        <v>51447</v>
       </c>
       <c r="G85" t="n">
         <v>15774.57</v>
@@ -3027,7 +3027,7 @@
         <v>105</v>
       </c>
       <c r="F93" t="n">
-        <v>17262</v>
+        <v>17260</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -3055,7 +3055,7 @@
         <v>73</v>
       </c>
       <c r="F94" t="n">
-        <v>26638</v>
+        <v>26635</v>
       </c>
       <c r="G94" t="n">
         <v>3176.27</v>
@@ -3254,10 +3254,10 @@
         <v>11750</v>
       </c>
       <c r="G101" t="n">
-        <v>15246.62</v>
+        <v>16940.69</v>
       </c>
       <c r="H101" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102">
@@ -3301,13 +3301,13 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>5358.04</v>
+        <v>5350.469999999999</v>
       </c>
       <c r="E103" t="n">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F103" t="n">
-        <v>119150</v>
+        <v>119146</v>
       </c>
       <c r="G103" t="n">
         <v>27105.12</v>
@@ -3363,13 +3363,13 @@
         <v>227</v>
       </c>
       <c r="F105" t="n">
-        <v>45575</v>
+        <v>45573</v>
       </c>
       <c r="G105" t="n">
-        <v>10186.44</v>
+        <v>11202.54</v>
       </c>
       <c r="H105" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106">
@@ -3391,13 +3391,13 @@
         <v>114</v>
       </c>
       <c r="F106" t="n">
-        <v>33059</v>
+        <v>33058</v>
       </c>
       <c r="G106" t="n">
-        <v>3056.78</v>
+        <v>4072.88</v>
       </c>
       <c r="H106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="107">
@@ -3553,13 +3553,13 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>6557.42</v>
+        <v>6554.33</v>
       </c>
       <c r="E112" t="n">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="F112" t="n">
-        <v>85064</v>
+        <v>85063</v>
       </c>
       <c r="G112" t="n">
         <v>27321.15</v>
@@ -3674,10 +3674,10 @@
         <v>91663</v>
       </c>
       <c r="G116" t="n">
-        <v>107289.04</v>
+        <v>110508.53</v>
       </c>
       <c r="H116" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="117">
@@ -3702,10 +3702,10 @@
         <v>52702</v>
       </c>
       <c r="G117" t="n">
-        <v>46433.92</v>
+        <v>52365.28</v>
       </c>
       <c r="H117" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="118">
@@ -3923,7 +3923,7 @@
         <v>13</v>
       </c>
       <c r="F125" t="n">
-        <v>5231</v>
+        <v>5228</v>
       </c>
       <c r="G125" t="n">
         <v>0</v>
@@ -4063,7 +4063,7 @@
         <v>141</v>
       </c>
       <c r="F130" t="n">
-        <v>8525</v>
+        <v>8524</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
@@ -4091,7 +4091,7 @@
         <v>72</v>
       </c>
       <c r="F131" t="n">
-        <v>5771</v>
+        <v>5770</v>
       </c>
       <c r="G131" t="n">
         <v>0</v>
@@ -4119,7 +4119,7 @@
         <v>56</v>
       </c>
       <c r="F132" t="n">
-        <v>5667</v>
+        <v>5666</v>
       </c>
       <c r="G132" t="n">
         <v>0</v>
@@ -4147,7 +4147,7 @@
         <v>44</v>
       </c>
       <c r="F133" t="n">
-        <v>6291</v>
+        <v>6290</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
@@ -4315,7 +4315,7 @@
         <v>37</v>
       </c>
       <c r="F139" t="n">
-        <v>14024</v>
+        <v>14023</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
@@ -4343,13 +4343,13 @@
         <v>225</v>
       </c>
       <c r="F140" t="n">
-        <v>67468</v>
+        <v>67457</v>
       </c>
       <c r="G140" t="n">
-        <v>823.73</v>
+        <v>5399.15</v>
       </c>
       <c r="H140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141">
@@ -4371,7 +4371,7 @@
         <v>84</v>
       </c>
       <c r="F141" t="n">
-        <v>19633</v>
+        <v>19630</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
@@ -4794,7 +4794,7 @@
         <v>5283</v>
       </c>
       <c r="G156" t="n">
-        <v>7283.9</v>
+        <v>7283.89</v>
       </c>
       <c r="H156" t="n">
         <v>5</v>
@@ -5127,7 +5127,7 @@
         <v>112</v>
       </c>
       <c r="F168" t="n">
-        <v>22815</v>
+        <v>22814</v>
       </c>
       <c r="G168" t="n">
         <v>0</v>
@@ -5155,7 +5155,7 @@
         <v>109</v>
       </c>
       <c r="F169" t="n">
-        <v>84151</v>
+        <v>84148</v>
       </c>
       <c r="G169" t="n">
         <v>4506.780000000001</v>
@@ -5183,7 +5183,7 @@
         <v>37</v>
       </c>
       <c r="F170" t="n">
-        <v>12244</v>
+        <v>12243</v>
       </c>
       <c r="G170" t="n">
         <v>2244.92</v>
@@ -5211,7 +5211,7 @@
         <v>21</v>
       </c>
       <c r="F171" t="n">
-        <v>12288</v>
+        <v>12287</v>
       </c>
       <c r="G171" t="n">
         <v>11692.38</v>
@@ -5295,7 +5295,7 @@
         <v>9</v>
       </c>
       <c r="F174" t="n">
-        <v>3764</v>
+        <v>3763</v>
       </c>
       <c r="G174" t="n">
         <v>0</v>
@@ -5345,13 +5345,13 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>133.11</v>
+        <v>129.59</v>
       </c>
       <c r="E176" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F176" t="n">
-        <v>5495</v>
+        <v>5494</v>
       </c>
       <c r="G176" t="n">
         <v>6777.96</v>
@@ -5519,7 +5519,7 @@
         <v>819</v>
       </c>
       <c r="F182" t="n">
-        <v>69367</v>
+        <v>69366</v>
       </c>
       <c r="G182" t="n">
         <v>12538.15</v>
@@ -5715,7 +5715,7 @@
         <v>948</v>
       </c>
       <c r="F189" t="n">
-        <v>155689</v>
+        <v>155685</v>
       </c>
       <c r="G189" t="n">
         <v>8624.58</v>
@@ -5827,7 +5827,7 @@
         <v>22</v>
       </c>
       <c r="F193" t="n">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="G193" t="n">
         <v>1355.08</v>
@@ -5970,10 +5970,10 @@
         <v>28034</v>
       </c>
       <c r="G198" t="n">
-        <v>18385.58</v>
+        <v>21647.44</v>
       </c>
       <c r="H198" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="199">
@@ -6051,7 +6051,7 @@
         <v>29</v>
       </c>
       <c r="F201" t="n">
-        <v>6000</v>
+        <v>5998</v>
       </c>
       <c r="G201" t="n">
         <v>0</v>
@@ -6219,7 +6219,7 @@
         <v>119</v>
       </c>
       <c r="F207" t="n">
-        <v>22310</v>
+        <v>22308</v>
       </c>
       <c r="G207" t="n">
         <v>2626.27</v>
@@ -6247,7 +6247,7 @@
         <v>215</v>
       </c>
       <c r="F208" t="n">
-        <v>49229</v>
+        <v>49225</v>
       </c>
       <c r="G208" t="n">
         <v>9527.969999999999</v>
@@ -6275,7 +6275,7 @@
         <v>134</v>
       </c>
       <c r="F209" t="n">
-        <v>21168</v>
+        <v>21166</v>
       </c>
       <c r="G209" t="n">
         <v>4066.95</v>
@@ -6303,7 +6303,7 @@
         <v>5</v>
       </c>
       <c r="F210" t="n">
-        <v>5904</v>
+        <v>5903</v>
       </c>
       <c r="G210" t="n">
         <v>0</v>
@@ -6499,7 +6499,7 @@
         <v>24</v>
       </c>
       <c r="F217" t="n">
-        <v>4935</v>
+        <v>4934</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -6555,7 +6555,7 @@
         <v>11</v>
       </c>
       <c r="F219" t="n">
-        <v>2086</v>
+        <v>2085</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
@@ -6639,7 +6639,7 @@
         <v>83</v>
       </c>
       <c r="F222" t="n">
-        <v>10144</v>
+        <v>10142</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
@@ -6779,7 +6779,7 @@
         <v>156</v>
       </c>
       <c r="F227" t="n">
-        <v>24773</v>
+        <v>24772</v>
       </c>
       <c r="G227" t="n">
         <v>3925.44</v>
@@ -6807,13 +6807,13 @@
         <v>380</v>
       </c>
       <c r="F228" t="n">
-        <v>62364</v>
+        <v>62361</v>
       </c>
       <c r="G228" t="n">
-        <v>0</v>
+        <v>7033.05</v>
       </c>
       <c r="H228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="229">
@@ -6863,7 +6863,7 @@
         <v>291</v>
       </c>
       <c r="F230" t="n">
-        <v>54571</v>
+        <v>54570</v>
       </c>
       <c r="G230" t="n">
         <v>5080.5</v>
@@ -6891,7 +6891,7 @@
         <v>217</v>
       </c>
       <c r="F231" t="n">
-        <v>61693</v>
+        <v>61692</v>
       </c>
       <c r="G231" t="n">
         <v>1694.07</v>
@@ -6919,7 +6919,7 @@
         <v>10</v>
       </c>
       <c r="F232" t="n">
-        <v>3043</v>
+        <v>3042</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -7031,7 +7031,7 @@
         <v>39</v>
       </c>
       <c r="F236" t="n">
-        <v>11075</v>
+        <v>11074</v>
       </c>
       <c r="G236" t="n">
         <v>4066.95</v>
@@ -7059,7 +7059,7 @@
         <v>25</v>
       </c>
       <c r="F237" t="n">
-        <v>3282</v>
+        <v>3281</v>
       </c>
       <c r="G237" t="n">
         <v>7879.66</v>
@@ -7115,7 +7115,7 @@
         <v>30</v>
       </c>
       <c r="F239" t="n">
-        <v>3430</v>
+        <v>3429</v>
       </c>
       <c r="G239" t="n">
         <v>2668.64</v>
@@ -7395,13 +7395,13 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>8553</v>
+        <v>8552</v>
       </c>
       <c r="G249" t="n">
-        <v>3768.65</v>
+        <v>2074.58</v>
       </c>
       <c r="H249" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="250">
@@ -7535,7 +7535,7 @@
         <v>67</v>
       </c>
       <c r="F254" t="n">
-        <v>6115</v>
+        <v>6114</v>
       </c>
       <c r="G254" t="n">
         <v>0</v>
@@ -7787,7 +7787,7 @@
         <v>1662</v>
       </c>
       <c r="F263" t="n">
-        <v>174846</v>
+        <v>174844</v>
       </c>
       <c r="G263" t="n">
         <v>21382.17</v>
@@ -7871,7 +7871,7 @@
         <v>387</v>
       </c>
       <c r="F266" t="n">
-        <v>31163</v>
+        <v>31162</v>
       </c>
       <c r="G266" t="n">
         <v>22283.9</v>
@@ -7899,7 +7899,7 @@
         <v>898</v>
       </c>
       <c r="F267" t="n">
-        <v>101560</v>
+        <v>101558</v>
       </c>
       <c r="G267" t="n">
         <v>14066.1</v>
@@ -8039,7 +8039,7 @@
         <v>247</v>
       </c>
       <c r="F272" t="n">
-        <v>21789</v>
+        <v>21788</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -8095,7 +8095,7 @@
         <v>1803</v>
       </c>
       <c r="F274" t="n">
-        <v>171007</v>
+        <v>171005</v>
       </c>
       <c r="G274" t="n">
         <v>34740.69</v>
@@ -8431,7 +8431,7 @@
         <v>456</v>
       </c>
       <c r="F286" t="n">
-        <v>16849</v>
+        <v>16848</v>
       </c>
       <c r="G286" t="n">
         <v>18976.25</v>
@@ -8459,7 +8459,7 @@
         <v>320</v>
       </c>
       <c r="F287" t="n">
-        <v>17795</v>
+        <v>17794</v>
       </c>
       <c r="G287" t="n">
         <v>30333.91</v>
@@ -8487,7 +8487,7 @@
         <v>475</v>
       </c>
       <c r="F288" t="n">
-        <v>34194</v>
+        <v>34193</v>
       </c>
       <c r="G288" t="n">
         <v>32283.05</v>
@@ -8515,7 +8515,7 @@
         <v>196</v>
       </c>
       <c r="F289" t="n">
-        <v>25467</v>
+        <v>25466</v>
       </c>
       <c r="G289" t="n">
         <v>22455.09</v>
@@ -8879,7 +8879,7 @@
         <v>50</v>
       </c>
       <c r="F302" t="n">
-        <v>15135</v>
+        <v>15134</v>
       </c>
       <c r="G302" t="n">
         <v>3410.16</v>
@@ -9243,7 +9243,7 @@
         <v>10</v>
       </c>
       <c r="F315" t="n">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -9411,13 +9411,13 @@
         <v>22</v>
       </c>
       <c r="F321" t="n">
-        <v>2947</v>
+        <v>2946</v>
       </c>
       <c r="G321" t="n">
-        <v>0</v>
+        <v>3982.2</v>
       </c>
       <c r="H321" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="322">
@@ -9439,7 +9439,7 @@
         <v>17</v>
       </c>
       <c r="F322" t="n">
-        <v>2337</v>
+        <v>2336</v>
       </c>
       <c r="G322" t="n">
         <v>0</v>
@@ -9747,7 +9747,7 @@
         <v>77</v>
       </c>
       <c r="F333" t="n">
-        <v>12721</v>
+        <v>12720</v>
       </c>
       <c r="G333" t="n">
         <v>8814.4</v>
@@ -10058,10 +10058,10 @@
         <v>15774</v>
       </c>
       <c r="G344" t="n">
-        <v>4950.85</v>
+        <v>5500.85</v>
       </c>
       <c r="H344" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="345">
@@ -10251,7 +10251,7 @@
         <v>451</v>
       </c>
       <c r="F351" t="n">
-        <v>57501</v>
+        <v>57499</v>
       </c>
       <c r="G351" t="n">
         <v>26004.27</v>
@@ -10674,10 +10674,10 @@
         <v>131352</v>
       </c>
       <c r="G366" t="n">
-        <v>49859.78</v>
+        <v>56594.54</v>
       </c>
       <c r="H366" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="367">
@@ -10811,7 +10811,7 @@
         <v>592</v>
       </c>
       <c r="F371" t="n">
-        <v>107326</v>
+        <v>107324</v>
       </c>
       <c r="G371" t="n">
         <v>7112.700000000001</v>
@@ -10979,7 +10979,7 @@
         <v>11</v>
       </c>
       <c r="F377" t="n">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="G377" t="n">
         <v>0</v>
@@ -11651,7 +11651,7 @@
         <v>9</v>
       </c>
       <c r="F401" t="n">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="G401" t="n">
         <v>2244.92</v>
@@ -11679,7 +11679,7 @@
         <v>8</v>
       </c>
       <c r="F402" t="n">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="G402" t="n">
         <v>0</v>
@@ -12519,7 +12519,7 @@
         <v>1</v>
       </c>
       <c r="F432" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G432" t="n">
         <v>0</v>
@@ -12687,7 +12687,7 @@
         <v>2</v>
       </c>
       <c r="F438" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G438" t="n">
         <v>0</v>
@@ -12855,7 +12855,7 @@
         <v>2</v>
       </c>
       <c r="F444" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G444" t="n">
         <v>0</v>
@@ -13107,7 +13107,7 @@
         <v>14</v>
       </c>
       <c r="F453" t="n">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="G453" t="n">
         <v>0</v>
@@ -13191,7 +13191,7 @@
         <v>17</v>
       </c>
       <c r="F456" t="n">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="G456" t="n">
         <v>2668.64</v>
@@ -13247,7 +13247,7 @@
         <v>13</v>
       </c>
       <c r="F458" t="n">
-        <v>2486</v>
+        <v>2485</v>
       </c>
       <c r="G458" t="n">
         <v>0</v>
@@ -13275,7 +13275,7 @@
         <v>0</v>
       </c>
       <c r="F459" t="n">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="G459" t="n">
         <v>0</v>
@@ -13303,7 +13303,7 @@
         <v>0</v>
       </c>
       <c r="F460" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G460" t="n">
         <v>0</v>
@@ -13779,7 +13779,7 @@
         <v>1</v>
       </c>
       <c r="F477" t="n">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="G477" t="n">
         <v>0</v>
@@ -13807,7 +13807,7 @@
         <v>72</v>
       </c>
       <c r="F478" t="n">
-        <v>5073</v>
+        <v>5072</v>
       </c>
       <c r="G478" t="n">
         <v>4955.93</v>
@@ -14059,7 +14059,7 @@
         <v>4</v>
       </c>
       <c r="F487" t="n">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G487" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>7626.27</v>
       </c>
       <c r="H495" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="496">
@@ -14871,7 +14871,7 @@
         <v>9</v>
       </c>
       <c r="F516" t="n">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="G516" t="n">
         <v>3727.97</v>
@@ -15089,13 +15089,13 @@
         </is>
       </c>
       <c r="D524" t="n">
-        <v>742.6800000000001</v>
+        <v>737.65</v>
       </c>
       <c r="E524" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F524" t="n">
-        <v>19076</v>
+        <v>19075</v>
       </c>
       <c r="G524" t="n">
         <v>6776.28</v>
@@ -15207,7 +15207,7 @@
         <v>128</v>
       </c>
       <c r="F528" t="n">
-        <v>25703</v>
+        <v>25701</v>
       </c>
       <c r="G528" t="n">
         <v>7457.48</v>
@@ -15319,7 +15319,7 @@
         <v>87</v>
       </c>
       <c r="F532" t="n">
-        <v>28921</v>
+        <v>28919</v>
       </c>
       <c r="G532" t="n">
         <v>0</v>
@@ -15406,10 +15406,10 @@
         <v>8443</v>
       </c>
       <c r="G535" t="n">
-        <v>7370.34</v>
+        <v>9445.76</v>
       </c>
       <c r="H535" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="536">
@@ -15431,7 +15431,7 @@
         <v>7</v>
       </c>
       <c r="F536" t="n">
-        <v>4103</v>
+        <v>4102</v>
       </c>
       <c r="G536" t="n">
         <v>0</v>
@@ -15515,7 +15515,7 @@
         <v>26</v>
       </c>
       <c r="F539" t="n">
-        <v>13159</v>
+        <v>13158</v>
       </c>
       <c r="G539" t="n">
         <v>0</v>
@@ -15655,7 +15655,7 @@
         <v>19</v>
       </c>
       <c r="F544" t="n">
-        <v>4562</v>
+        <v>4561</v>
       </c>
       <c r="G544" t="n">
         <v>2456.78</v>
@@ -15711,7 +15711,7 @@
         <v>41</v>
       </c>
       <c r="F546" t="n">
-        <v>11028</v>
+        <v>11026</v>
       </c>
       <c r="G546" t="n">
         <v>0</v>
@@ -15808,7 +15808,7 @@
       <c r="A550" t="inlineStr"/>
       <c r="B550" t="inlineStr">
         <is>
-          <t>AudioArray_Wireless Mic_SP_KT/PT</t>
+          <t>AudioArray_Wireless Mic_SP_KT</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
@@ -16019,7 +16019,7 @@
         <v>849</v>
       </c>
       <c r="F5" t="n">
-        <v>241206</v>
+        <v>241174</v>
       </c>
       <c r="G5" t="n">
         <v>28468.65</v>
@@ -16041,10 +16041,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1743.99</v>
+        <v>1740.8</v>
       </c>
       <c r="E6" t="n">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F6" t="n">
         <v>52921</v>
@@ -16246,10 +16246,10 @@
         <v>98791</v>
       </c>
       <c r="G13" t="n">
-        <v>25585.6</v>
+        <v>29652.55</v>
       </c>
       <c r="H13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -16834,10 +16834,10 @@
         <v>136999</v>
       </c>
       <c r="G34" t="n">
-        <v>35905.06</v>
+        <v>39547.43</v>
       </c>
       <c r="H34" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -16965,13 +16965,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9689.809999999999</v>
+        <v>9681.91</v>
       </c>
       <c r="E39" t="n">
-        <v>4690</v>
+        <v>4683</v>
       </c>
       <c r="F39" t="n">
-        <v>1303555</v>
+        <v>1303551</v>
       </c>
       <c r="G39" t="n">
         <v>39993.23</v>
@@ -17111,13 +17111,13 @@
         <v>426</v>
       </c>
       <c r="F44" t="n">
-        <v>124926</v>
+        <v>124921</v>
       </c>
       <c r="G44" t="n">
-        <v>21898.35</v>
+        <v>24166.15</v>
       </c>
       <c r="H44" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45">
@@ -17159,7 +17159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17255,19 +17255,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4789</v>
+        <v>9232</v>
       </c>
       <c r="E3" t="n">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>917.6499887013158</v>
+        <v>1768.966666666666</v>
       </c>
       <c r="G3" t="n">
-        <v>1928.01774558022</v>
+        <v>3716.666666666667</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -17288,19 +17288,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>13040</v>
+        <v>9232</v>
       </c>
       <c r="E4" t="n">
-        <v>151</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>2498.443292284613</v>
+        <v>1768.966666666666</v>
       </c>
       <c r="G4" t="n">
-        <v>5249.324974839065</v>
+        <v>3716.666666666667</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -17321,19 +17321,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>8578</v>
+        <v>9232</v>
       </c>
       <c r="E5" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="F5" t="n">
-        <v>1643.565905888608</v>
+        <v>1768.966666666666</v>
       </c>
       <c r="G5" t="n">
-        <v>3453.194869068191</v>
+        <v>3716.666666666667</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -17345,28 +17345,28 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Audio Array-B0BLJVJ2GN-AA 05 Suspension-SB-PT</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Audio Interface-SBV -PT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>B0DT6T6N6B</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1290</v>
+        <v>86255</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>650</v>
       </c>
       <c r="F6" t="n">
-        <v>247.2408131254628</v>
+        <v>6314.280000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>519.4624105125235</v>
+        <v>26773.73</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -17378,28 +17378,28 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Audio Interface-SBV -PT</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-KT-Phrase</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>75886</v>
+        <v>63583</v>
       </c>
       <c r="E7" t="n">
-        <v>557</v>
+        <v>333</v>
       </c>
       <c r="F7" t="n">
-        <v>5438.830627693358</v>
+        <v>4585.87</v>
       </c>
       <c r="G7" t="n">
-        <v>23077.74380074495</v>
+        <v>16777.11</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -17411,28 +17411,28 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Audio Interface-SBV -PT</t>
+          <t>Audio Array-B0DXFPM4N2-Studio Monitor- SBV-CT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0DXFPM4N2</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10371</v>
+        <v>24326</v>
       </c>
       <c r="E8" t="n">
-        <v>94</v>
+        <v>288</v>
       </c>
       <c r="F8" t="n">
-        <v>878.5893723066407</v>
+        <v>2888.37</v>
       </c>
       <c r="G8" t="n">
-        <v>3695.986199255054</v>
+        <v>21607.62</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -17444,28 +17444,28 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-KT-Phrase</t>
+          <t>Audio Array-Catch All-Condenser -SB-PT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B0BLKBJ5HN</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>30187</v>
+        <v>13232</v>
       </c>
       <c r="E9" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F9" t="n">
-        <v>2177.228439075621</v>
+        <v>3506.613333333333</v>
       </c>
       <c r="G9" t="n">
-        <v>7965.25</v>
+        <v>11366.11666666667</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -17477,28 +17477,28 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-KT-Phrase</t>
+          <t>Audio Array-Catch All-Condenser -SB-PT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0D3M1B4Z8</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>33396</v>
+        <v>13232</v>
       </c>
       <c r="E10" t="n">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="F10" t="n">
-        <v>2408.641560924379</v>
+        <v>3506.613333333333</v>
       </c>
       <c r="G10" t="n">
-        <v>8811.860000000001</v>
+        <v>11366.11666666667</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -17510,28 +17510,28 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Audio Array-B0DXFPM4N2-Studio Monitor- SBV-CT</t>
+          <t>Audio Array-Catch All-Condenser -SB-PT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B0DXFPM4N2</t>
+          <t>B0FF9R3GKK</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10785</v>
+        <v>13232</v>
       </c>
       <c r="E11" t="n">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="F11" t="n">
-        <v>1280.542172304</v>
+        <v>3506.613333333333</v>
       </c>
       <c r="G11" t="n">
-        <v>9579.613641299196</v>
+        <v>11366.11666666667</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -17543,28 +17543,28 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Audio Array-B0DXFPM4N2-Studio Monitor- SBV-CT</t>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B0G3B677Z5</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13541</v>
+        <v>8276</v>
       </c>
       <c r="E12" t="n">
-        <v>160</v>
+        <v>44</v>
       </c>
       <c r="F12" t="n">
-        <v>1607.827827695999</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G12" t="n">
-        <v>12028.0063587008</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -17576,28 +17576,28 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Condenser -SB-PT</t>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0B4DS678Q</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>25260</v>
+        <v>8276</v>
       </c>
       <c r="E13" t="n">
-        <v>307</v>
+        <v>44</v>
       </c>
       <c r="F13" t="n">
-        <v>6694.218635372819</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G13" t="n">
-        <v>20269.6832562609</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -17609,7 +17609,7 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Condenser -SB-PT</t>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -17618,19 +17618,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5175</v>
+        <v>8276</v>
       </c>
       <c r="E14" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F14" t="n">
-        <v>1371.475531701826</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G14" t="n">
-        <v>4152.743753305837</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -17642,28 +17642,28 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Condenser -SB-PT</t>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B0D3M1B4Z8</t>
+          <t>B0B4G1PXWV</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9260</v>
+        <v>8276</v>
       </c>
       <c r="E15" t="n">
-        <v>113</v>
+        <v>44</v>
       </c>
       <c r="F15" t="n">
-        <v>2454.145832925355</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G15" t="n">
-        <v>7431.002990433267</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -17680,23 +17680,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0B4G89VQJ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>17484</v>
+        <v>8276</v>
       </c>
       <c r="E16" t="n">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F16" t="n">
-        <v>928.322822742556</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G16" t="n">
-        <v>8979.68</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -17713,20 +17713,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0B4JRQP22</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6268</v>
+        <v>8276</v>
       </c>
       <c r="E17" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="F17" t="n">
-        <v>332.8321326140165</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G17" t="n">
-        <v>3219.49</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
@@ -17750,16 +17750,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7182</v>
+        <v>8276</v>
       </c>
       <c r="E18" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F18" t="n">
-        <v>355.3103836171088</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G18" t="n">
-        <v>3388.98</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H18" t="n">
         <v>1</v>
@@ -17783,16 +17783,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4218</v>
+        <v>8276</v>
       </c>
       <c r="E19" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="F19" t="n">
-        <v>208.7086009533565</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G19" t="n">
-        <v>1990.68</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H19" t="n">
         <v>1</v>
@@ -17816,19 +17816,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9005</v>
+        <v>8276</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="F20" t="n">
-        <v>1751.148729970681</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G20" t="n">
-        <v>2212.886641673554</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -17845,23 +17845,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0BLK8DNPD</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>145604</v>
+        <v>8276</v>
       </c>
       <c r="E21" t="n">
-        <v>622</v>
+        <v>44</v>
       </c>
       <c r="F21" t="n">
-        <v>7698.42</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G21" t="n">
-        <v>26519.49</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H21" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -17878,23 +17878,23 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>B0BQ7H7418</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9012</v>
+        <v>8276</v>
       </c>
       <c r="E22" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="F22" t="n">
-        <v>1752.501890352931</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G22" t="n">
-        <v>2214.596599533029</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -17911,23 +17911,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0C4YTNJG7</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28010</v>
+        <v>8276</v>
       </c>
       <c r="E23" t="n">
-        <v>191</v>
+        <v>44</v>
       </c>
       <c r="F23" t="n">
-        <v>1385.791015429535</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G23" t="n">
-        <v>13217.79</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -17944,23 +17944,23 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>B0DT6T6N6B</t>
+          <t>B0C539RBGL</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8034</v>
+        <v>8276</v>
       </c>
       <c r="E24" t="n">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="F24" t="n">
-        <v>1562.279379676389</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G24" t="n">
-        <v>1974.216758793417</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -17977,25 +17977,520 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>B0FJ8TSQK1</t>
+          <t>B0CF5R3V95</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5196</v>
+        <v>8276</v>
       </c>
       <c r="E25" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="F25" t="n">
-        <v>275.8850446434276</v>
+        <v>560.3862068965518</v>
       </c>
       <c r="G25" t="n">
-        <v>2668.64</v>
+        <v>2289.187931034483</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>B0CF5RRTDJ</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E26" t="n">
+        <v>44</v>
+      </c>
+      <c r="F26" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>B0CF5TCQKL</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E27" t="n">
+        <v>44</v>
+      </c>
+      <c r="F27" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>B0CH4RT4P8</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E28" t="n">
+        <v>44</v>
+      </c>
+      <c r="F28" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E29" t="n">
+        <v>44</v>
+      </c>
+      <c r="F29" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>B0CM6NTWBP</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E30" t="n">
+        <v>44</v>
+      </c>
+      <c r="F30" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>B0D3M1B4Z8</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E31" t="n">
+        <v>44</v>
+      </c>
+      <c r="F31" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>B0DFMLS8JG</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E32" t="n">
+        <v>44</v>
+      </c>
+      <c r="F32" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>B0DFMMTWLY</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E33" t="n">
+        <v>44</v>
+      </c>
+      <c r="F33" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>B0DFMNGFTD</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E34" t="n">
+        <v>44</v>
+      </c>
+      <c r="F34" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>B0DT6T6N6B</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E35" t="n">
+        <v>44</v>
+      </c>
+      <c r="F35" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>B0FF9R3GKK</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E36" t="n">
+        <v>44</v>
+      </c>
+      <c r="F36" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>B0G2C2RCXN</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E37" t="n">
+        <v>44</v>
+      </c>
+      <c r="F37" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>B0G3Q517Y2</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E38" t="n">
+        <v>44</v>
+      </c>
+      <c r="F38" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>B0G3Q59X8C</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E39" t="n">
+        <v>44</v>
+      </c>
+      <c r="F39" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>B0G4DNF8RZ</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>8276</v>
+      </c>
+      <c r="E40" t="n">
+        <v>44</v>
+      </c>
+      <c r="F40" t="n">
+        <v>560.3862068965518</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2289.187931034483</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
         <is>
           <t>Audio Array</t>
         </is>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-06-07
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week22.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week22.xlsx
@@ -787,7 +787,7 @@
         <v>42</v>
       </c>
       <c r="F13" t="n">
-        <v>12187</v>
+        <v>12186</v>
       </c>
       <c r="G13" t="n">
         <v>8471.200000000001</v>
@@ -1039,7 +1039,7 @@
         <v>155</v>
       </c>
       <c r="F22" t="n">
-        <v>28485</v>
+        <v>28484</v>
       </c>
       <c r="G22" t="n">
         <v>9615.25</v>
@@ -1263,7 +1263,7 @@
         <v>206</v>
       </c>
       <c r="F30" t="n">
-        <v>23072</v>
+        <v>23070</v>
       </c>
       <c r="G30" t="n">
         <v>13486.46</v>
@@ -1711,7 +1711,7 @@
         <v>86</v>
       </c>
       <c r="F46" t="n">
-        <v>26089</v>
+        <v>26086</v>
       </c>
       <c r="G46" t="n">
         <v>1647.46</v>
@@ -3195,7 +3195,7 @@
         <v>120</v>
       </c>
       <c r="F99" t="n">
-        <v>8816</v>
+        <v>8815</v>
       </c>
       <c r="G99" t="n">
         <v>14739.84</v>
@@ -5295,7 +5295,7 @@
         <v>4</v>
       </c>
       <c r="F174" t="n">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="G174" t="n">
         <v>0</v>
@@ -5323,7 +5323,7 @@
         <v>41</v>
       </c>
       <c r="F175" t="n">
-        <v>15490</v>
+        <v>15489</v>
       </c>
       <c r="G175" t="n">
         <v>823.73</v>
@@ -5463,7 +5463,7 @@
         <v>20</v>
       </c>
       <c r="F180" t="n">
-        <v>17093</v>
+        <v>17092</v>
       </c>
       <c r="G180" t="n">
         <v>1100</v>
@@ -5575,7 +5575,7 @@
         <v>841</v>
       </c>
       <c r="F184" t="n">
-        <v>136376</v>
+        <v>136374</v>
       </c>
       <c r="G184" t="n">
         <v>8624.58</v>
@@ -5743,7 +5743,7 @@
         <v>26</v>
       </c>
       <c r="F190" t="n">
-        <v>31060</v>
+        <v>31059</v>
       </c>
       <c r="G190" t="n">
         <v>0</v>
@@ -5771,7 +5771,7 @@
         <v>13</v>
       </c>
       <c r="F191" t="n">
-        <v>1632</v>
+        <v>1631</v>
       </c>
       <c r="G191" t="n">
         <v>0</v>
@@ -6079,7 +6079,7 @@
         <v>85</v>
       </c>
       <c r="F202" t="n">
-        <v>15820</v>
+        <v>15819</v>
       </c>
       <c r="G202" t="n">
         <v>2626.27</v>
@@ -6639,7 +6639,7 @@
         <v>134</v>
       </c>
       <c r="F222" t="n">
-        <v>21457</v>
+        <v>21456</v>
       </c>
       <c r="G222" t="n">
         <v>2453.4</v>
@@ -6667,7 +6667,7 @@
         <v>294</v>
       </c>
       <c r="F223" t="n">
-        <v>49875</v>
+        <v>49874</v>
       </c>
       <c r="G223" t="n">
         <v>7033.05</v>
@@ -6723,7 +6723,7 @@
         <v>258</v>
       </c>
       <c r="F225" t="n">
-        <v>51411</v>
+        <v>51410</v>
       </c>
       <c r="G225" t="n">
         <v>4064.4</v>
@@ -6751,7 +6751,7 @@
         <v>195</v>
       </c>
       <c r="F226" t="n">
-        <v>54951</v>
+        <v>54950</v>
       </c>
       <c r="G226" t="n">
         <v>1694.07</v>
@@ -6891,7 +6891,7 @@
         <v>35</v>
       </c>
       <c r="F231" t="n">
-        <v>9581</v>
+        <v>9580</v>
       </c>
       <c r="G231" t="n">
         <v>4066.95</v>
@@ -7311,7 +7311,7 @@
         <v>55</v>
       </c>
       <c r="F246" t="n">
-        <v>20667</v>
+        <v>20666</v>
       </c>
       <c r="G246" t="n">
         <v>1694.07</v>
@@ -7647,7 +7647,7 @@
         <v>1469</v>
       </c>
       <c r="F258" t="n">
-        <v>160041</v>
+        <v>160040</v>
       </c>
       <c r="G258" t="n">
         <v>16638.11</v>
@@ -7759,7 +7759,7 @@
         <v>786</v>
       </c>
       <c r="F262" t="n">
-        <v>91431</v>
+        <v>91430</v>
       </c>
       <c r="G262" t="n">
         <v>7033.05</v>
@@ -10055,7 +10055,7 @@
         <v>373</v>
       </c>
       <c r="F344" t="n">
-        <v>45784</v>
+        <v>45783</v>
       </c>
       <c r="G344" t="n">
         <v>24310.2</v>
@@ -10167,7 +10167,7 @@
         <v>50</v>
       </c>
       <c r="F348" t="n">
-        <v>9612</v>
+        <v>9611</v>
       </c>
       <c r="G348" t="n">
         <v>4939.15</v>
@@ -14899,7 +14899,7 @@
         <v>102</v>
       </c>
       <c r="F517" t="n">
-        <v>18005</v>
+        <v>18004</v>
       </c>
       <c r="G517" t="n">
         <v>6776.28</v>
@@ -16103,7 +16103,7 @@
         <v>130</v>
       </c>
       <c r="F15" t="n">
-        <v>43903</v>
+        <v>43902</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -16775,7 +16775,7 @@
         <v>3918</v>
       </c>
       <c r="F39" t="n">
-        <v>1103807</v>
+        <v>1103806</v>
       </c>
       <c r="G39" t="n">
         <v>34061.87</v>
@@ -16915,7 +16915,7 @@
         <v>379</v>
       </c>
       <c r="F44" t="n">
-        <v>111149</v>
+        <v>111148</v>
       </c>
       <c r="G44" t="n">
         <v>26833.95</v>
@@ -17563,10 +17563,10 @@
         <v>591.6591060937562</v>
       </c>
       <c r="G18" t="n">
-        <v>4914.857198145436</v>
+        <v>6088.54068993285</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -17596,7 +17596,7 @@
         <v>347.5393626751172</v>
       </c>
       <c r="G19" t="n">
-        <v>2886.977181099965</v>
+        <v>3576.396491167114</v>
       </c>
       <c r="H19" t="n">
         <v>1</v>
@@ -17728,7 +17728,7 @@
         <v>769.2015312311266</v>
       </c>
       <c r="G23" t="n">
-        <v>6389.6856207546</v>
+        <v>7915.562818900036</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>

</xml_diff>